<commit_message>
Docs: update to hybrid power/control architecture
Rewrite firmware and power docs to target the hybrid harvest+storage architecture (RAK3172, TPS61291, 100 F supercap) and clarify firmware requirements. FIRMWARE_NEXT_STEPS.md and POWER_SYSTEM_ANALYSIS.md were reworked to emphasize ADC_MONITOR, VBAT_OK, P-FET sensor gating and a charge-first power state machine; TODO entries updated to map tasks to RAK3172 signals. Block diagram switched from embedded mermaid to an authoritative image (Docs/pics/BlockDiagram.jpg) and small UI/styling improvements added to several HTML docs (BOM, Sensors, EnergyBudget, TODO) with legacy notices. Added Docs/build_block_diagram.py and updated docs generation commands; updated scripts and firmware_todo references accordingly. Overall these changes align documentation with the new system architecture and call out firmware work needed before release.
</commit_message>
<xml_diff>
--- a/Docs/SolarSensorSchematicRev2_BOM.xlsx
+++ b/Docs/SolarSensorSchematicRev2_BOM.xlsx
@@ -4820,7 +4820,7 @@
     <row r="2">
       <c r="A2" s="20" t="inlineStr">
         <is>
-          <t>Hardware supports automatic solar bring-up (BQ_EN, VBAT_OK, 0.22 F supercap). Current lora_myself_net firmware does not. Close every open task before calling firmware Rev2-ready. Detail: FIRMWARE_NEXT_STEPS.md · POWER_SYSTEM_ANALYSIS.md</t>
+          <t>Hardware supports hybrid bring-up (BQ25505 OR paths, 100 F LIC supercap, P-FET sensor gates). Block diagram: pics/BlockDiagram.jpg · FIRMWARE_NEXT_STEPS.md · POWER_SYSTEM_ANALYSIS.md</t>
         </is>
       </c>
     </row>
@@ -4884,22 +4884,22 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Assign BQ_EN to an RA-08 GPIO</t>
+          <t>Assign ADC_MONITOR and status inputs on RAK3172</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>BQ_EN exists on the schematic; firmware never drives it.</t>
+          <t>Hybrid block diagram defines ADC_MONITOR, VBAT_OK, BAT_GD, PRIM_STATUS; not wired in legacy RA-08 firmware.</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>Confirm which RA-08 pin connects to BQ_EN and the active level. Add CONFIG_BQ_EN_* to lora_config.h.</t>
+          <t>Map each net to RAK3172 GPIO/ADC in lora_config.h. Confirm divider ratio for 100 F · 3.8 V supercap.</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>lora_config.h · schematic Rev2</t>
+          <t>lora_config.h · hybrid PCB</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
@@ -4926,22 +4926,22 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Assign VBAT_OK to an RA-08 GPIO</t>
+          <t>Assign GPIO_RADAR and GPIO_CO2 P-FET gates</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>BQ25505 OK output is not read in firmware.</t>
+          <t>Radar and CO₂ use Si2301 P-FET gates; legacy firmware uses different RA-08 enables.</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Confirm VBAT_OK pin and polarity. Add CONFIG_VBAT_OK_* to lora_config.h.</t>
+          <t>Map GPIO_RADAR and GPIO_CO2 to RAK3172 outputs. Active level per hybrid schematic.</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>lora_config.h · schematic Rev2</t>
+          <t>lora_config.h · hybrid PCB</t>
         </is>
       </c>
       <c r="H6" s="30" t="inlineStr">
@@ -5010,17 +5010,17 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Drive BQ_EN during charge-only boot</t>
+          <t>Drive hybrid charge / path policy during boot</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>Harvester enable is floating or default; 0.22 F supercap may never charge correctly.</t>
+          <t>Harvester uses internal OR logic; firmware must not load gated sensors on flat 100 F supercap.</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Assert BQ_EN after first MCU wake. Keep all sensor enables off until vcap reaches target.</t>
+          <t>Implement charge-only boot: SHT41 only until ADC_MONITOR threshold; defer radar/CO₂ and LoRa TX.</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Add indoor solar docs and BQ25505 inputs
Add comprehensive indoor solar documentation and tooling for the Solar Sensor project: new BQ25505 design inputs, indoor solar panel spec, indoor solar cells HTML page, datasheets, ERC/report, schematic PDF, and supporting scripts (build_bq25505_tools.py, solar_cell_comparison.py). Update POWER_SYSTEM_ANALYSIS to include hybrid BQ25505 thresholds and references. Update BOM/HTML/XLSX and Energy Budget pages to reflect 60×60 mm panel sizing and note recommended ROV divider changes for 3.8 V LIC operation. Remove SESSION_CHECKPOINT.md and add .gitignore entries for local artifacts and pycache.
</commit_message>
<xml_diff>
--- a/Docs/SolarSensorSchematicRev2_BOM.xlsx
+++ b/Docs/SolarSensorSchematicRev2_BOM.xlsx
@@ -10,7 +10,8 @@
     <sheet name="BOM" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Energy Budget" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Power Optimization" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Firmware TODO" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Indoor Solar Cells" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Firmware TODO" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1882,7 +1883,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Harvesting threshold programming</t>
+          <t>Rev2 OVP network; hybrid 3.8V LIC: ROV1=4.02M — see BQ25505_DESIGN_INPUTS.md</t>
         </is>
       </c>
     </row>
@@ -1967,6 +1968,11 @@
       <c r="H28" t="inlineStr">
         <is>
           <t>7.32M 0805</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Rev2 OVP network; hybrid 3.8V LIC: ROV2=4.42M</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2906,7 @@
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
@@ -2909,7 +2915,7 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>40 mm × 40 mm</t>
+          <t>60×60 mm — Dazheng perovskite / indoor cell (vendor TBD)</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2935,7 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>Amorton-class @ ref lux</t>
+          <t>Placeholder until vendor curve; Amorton-class @ 200 lux</t>
         </is>
       </c>
     </row>
@@ -2949,7 +2955,7 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Indoor a-Si reference point</t>
+          <t>Indoor model point; deploy range 200–1000 lux</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3997,7 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>Indoor Solar — 40×40 mm Panel</t>
+          <t>Indoor Solar — 60×60 mm Panel</t>
         </is>
       </c>
       <c r="B60" s="27" t="n"/>
@@ -4797,6 +4803,1245 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Indoor Solar Cell Comparison — 60×60 mm (36 cm²) panel</t>
+        </is>
+      </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="27" t="n"/>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="27" t="n"/>
+      <c r="H1" s="27" t="n"/>
+      <c r="I1" s="28" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>Benchmark published indoor PV modules vs project load. Datasheets: datasheets/SolarCell/ · Dazheng target has no public electrical PDF. Test conditions vary (lux, spectrum, temp).</t>
+        </is>
+      </c>
+      <c r="B3" s="27" t="n"/>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="27" t="n"/>
+      <c r="E3" s="27" t="n"/>
+      <c r="F3" s="27" t="n"/>
+      <c r="G3" s="27" t="n"/>
+      <c r="H3" s="27" t="n"/>
+      <c r="I3" s="28" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Catalog @ 200 lux (scaled to 36 cm²)</t>
+        </is>
+      </c>
+      <c r="B5" s="27" t="n"/>
+      <c r="C5" s="27" t="n"/>
+      <c r="D5" s="27" t="n"/>
+      <c r="E5" s="27" t="n"/>
+      <c r="F5" s="27" t="n"/>
+      <c r="G5" s="27" t="n"/>
+      <c r="H5" s="27" t="n"/>
+      <c r="I5" s="28" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Native / catalog size</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>µW/cm² @ 200 lux</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Panel in (µW)</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Voc note</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Dazheng (target)</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Flexible perovskite 60×60</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Perovskite flexible</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>60×60 mm (custom)</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>TBD — request from vendor</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>INDOOR_SOLAR_PANEL_SPEC.md</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>Vendor under evaluation; no public electrical PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Epishine</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>MultiCell (typ max)</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Printed organic indoor</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>50×50 mm catalog; 60×60 custom</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>8.4</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>302</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>~0.5 V MPP/cell</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>datasheets/SolarCell/Epishine_MultiCell_indoor_datasheet.pdf</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>20–1000 lux SOC; 5000 K LED test conditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Panasonic</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Amorton (flyer typ)</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>a-Si indoor</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Custom sizes</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>288</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>~0.63 V/cell</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>datasheets/SolarCell/Panasonic_Amorton_product_flyer.pdf</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>7–9 µW/cm² @ 200 lux (fluorescent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Panasonic</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>AMG-1401C</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>a-Si indoor glass</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>41.4×26.1 mm</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>6.9</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>248</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>2.7 V Voc @ 200 lux FL</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>datasheets/SolarCell/Panasonic_AMG-1401C_indoor_datasheet.pdf</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>White fluorescent @ 200 lux</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>PowerFilm</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>LL200-2.4-37</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>a-Si flexible indoor</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>54×36.5 mm</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>~2.4 V Voc avg @ 200 lux</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>datasheets/SolarCell/PowerFilm_LL200-2.4-37_indoor_drawing.pdf</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>Closest catalog geometry to 60×60 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>RICOH</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>EH DSSC5284a</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Solid-state DSSC</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>52×84 mm</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>5.4 V Voc — check BQ25505 Vin</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>datasheets/SolarCell/RICOH_EH_DSSC5284a_launch_spec.pdf</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>200 lux, 5000 K LED; min Pmax rating</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Energy budget placeholder</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Amorton-class coeff</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>36 cm²</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>288</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>build_energy_budget_sheet.py</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>Replace when Dazheng sample is characterised</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Load reference (from Energy Budget sheet)</t>
+        </is>
+      </c>
+      <c r="B16" s="27" t="n"/>
+      <c r="C16" s="27" t="n"/>
+      <c r="D16" s="28" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Required net power (+ margin)</t>
+        </is>
+      </c>
+      <c r="B18" s="16">
+        <f>'Energy Budget'!B62</f>
+        <v/>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>µW</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Links to Energy Budget total × margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Harvester efficiency</t>
+        </is>
+      </c>
+      <c r="B19" s="10">
+        <f>'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="C19" s="10" t="inlineStr"/>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>BQ25505 end-to-end</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>@ 200 lux — panel input, harvested, vs budget</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="n"/>
+      <c r="C21" s="27" t="n"/>
+      <c r="D21" s="27" t="n"/>
+      <c r="E21" s="27" t="n"/>
+      <c r="F21" s="28" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Panel in (µW)</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Harvested (µW)</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>vs budget</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Dazheng (target)</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Flexible perovskite 60×60</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Epishine</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>MultiCell (typ max)</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="n">
+        <v>302.4</v>
+      </c>
+      <c r="D24" s="16">
+        <f>C24*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E24" s="16">
+        <f>D24/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F24" s="10">
+        <f>IF(D24&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Panasonic</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Amorton (flyer typ)</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="n">
+        <v>288</v>
+      </c>
+      <c r="D25" s="16">
+        <f>C25*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E25" s="16">
+        <f>D25/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F25" s="10">
+        <f>IF(D25&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Panasonic</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>AMG-1401C</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="n">
+        <v>247.5428952190572</v>
+      </c>
+      <c r="D26" s="16">
+        <f>C26*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E26" s="16">
+        <f>D26/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F26" s="10">
+        <f>IF(D26&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>PowerFilm</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>LL200-2.4-37</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="n">
+        <v>124.2009132420091</v>
+      </c>
+      <c r="D27" s="16">
+        <f>C27*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E27" s="16">
+        <f>D27/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F27" s="10">
+        <f>IF(D27&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>RICOH</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>EH DSSC5284a</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="n">
+        <v>227.4725274725275</v>
+      </c>
+      <c r="D28" s="16">
+        <f>C28*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E28" s="16">
+        <f>D28/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F28" s="10">
+        <f>IF(D28&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Energy budget placeholder</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="n">
+        <v>288</v>
+      </c>
+      <c r="D29" s="16">
+        <f>C29*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E29" s="16">
+        <f>D29/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F29" s="10">
+        <f>IF(D29&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>@ 500 lux — panel input, harvested, vs budget</t>
+        </is>
+      </c>
+      <c r="B31" s="27" t="n"/>
+      <c r="C31" s="27" t="n"/>
+      <c r="D31" s="27" t="n"/>
+      <c r="E31" s="27" t="n"/>
+      <c r="F31" s="28" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Panel in (µW)</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Harvested (µW)</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>vs budget</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Dazheng (target)</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Flexible perovskite 60×60</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Epishine</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>MultiCell (typ max)</t>
+        </is>
+      </c>
+      <c r="C34" s="16" t="n">
+        <v>756.0000000000001</v>
+      </c>
+      <c r="D34" s="16">
+        <f>C34*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E34" s="16">
+        <f>D34/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F34" s="10">
+        <f>IF(D34&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>Panasonic</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Amorton (flyer typ)</t>
+        </is>
+      </c>
+      <c r="C35" s="16" t="n">
+        <v>720</v>
+      </c>
+      <c r="D35" s="16">
+        <f>C35*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E35" s="16">
+        <f>D35/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F35" s="10">
+        <f>IF(D35&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Panasonic</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>AMG-1401C</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="n">
+        <v>618.8572380476429</v>
+      </c>
+      <c r="D36" s="16">
+        <f>C36*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E36" s="16">
+        <f>D36/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F36" s="10">
+        <f>IF(D36&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>PowerFilm</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>LL200-2.4-37</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="n">
+        <v>310.5022831050228</v>
+      </c>
+      <c r="D37" s="16">
+        <f>C37*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E37" s="16">
+        <f>D37/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F37" s="10">
+        <f>IF(D37&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>RICOH</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>EH DSSC5284a</t>
+        </is>
+      </c>
+      <c r="C38" s="16" t="n">
+        <v>568.6813186813187</v>
+      </c>
+      <c r="D38" s="16">
+        <f>C38*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E38" s="16">
+        <f>D38/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F38" s="10">
+        <f>IF(D38&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Energy budget placeholder</t>
+        </is>
+      </c>
+      <c r="C39" s="16" t="n">
+        <v>720</v>
+      </c>
+      <c r="D39" s="16">
+        <f>C39*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E39" s="16">
+        <f>D39/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F39" s="10">
+        <f>IF(D39&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>@ 1000 lux — panel input, harvested, vs budget</t>
+        </is>
+      </c>
+      <c r="B41" s="27" t="n"/>
+      <c r="C41" s="27" t="n"/>
+      <c r="D41" s="27" t="n"/>
+      <c r="E41" s="27" t="n"/>
+      <c r="F41" s="28" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Panel in (µW)</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>Harvested (µW)</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>vs budget</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>Dazheng (target)</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Flexible perovskite 60×60</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>Epishine</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>MultiCell (typ max)</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="n">
+        <v>1512</v>
+      </c>
+      <c r="D44" s="16">
+        <f>C44*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E44" s="16">
+        <f>D44/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F44" s="10">
+        <f>IF(D44&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>Panasonic</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Amorton (flyer typ)</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="n">
+        <v>1440</v>
+      </c>
+      <c r="D45" s="16">
+        <f>C45*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E45" s="16">
+        <f>D45/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F45" s="10">
+        <f>IF(D45&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>Panasonic</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>AMG-1401C</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="n">
+        <v>1237.714476095286</v>
+      </c>
+      <c r="D46" s="16">
+        <f>C46*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E46" s="16">
+        <f>D46/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F46" s="10">
+        <f>IF(D46&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>PowerFilm</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>LL200-2.4-37</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="n">
+        <v>621.0045662100456</v>
+      </c>
+      <c r="D47" s="16">
+        <f>C47*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E47" s="16">
+        <f>D47/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F47" s="10">
+        <f>IF(D47&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>RICOH</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>EH DSSC5284a</t>
+        </is>
+      </c>
+      <c r="C48" s="16" t="n">
+        <v>1137.362637362637</v>
+      </c>
+      <c r="D48" s="16">
+        <f>C48*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E48" s="16">
+        <f>D48/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F48" s="10">
+        <f>IF(D48&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>Energy budget placeholder</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="n">
+        <v>1440</v>
+      </c>
+      <c r="D49" s="16">
+        <f>C49*'Energy Budget'!$B$14</f>
+        <v/>
+      </c>
+      <c r="E49" s="16">
+        <f>D49/'Energy Budget'!$B$62</f>
+        <v/>
+      </c>
+      <c r="F49" s="10">
+        <f>IF(D49&gt;='Energy Budget'!$B$62,"OK","DEFICIT")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A21:F21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5062,7 +6307,7 @@
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>Measure droop during LoRa TX and sensor bursts. Set VCAP_MIN_TX_mV, VCAP_MIN_SENSORS_mV, VCAP_CHARGE_TARGET_mV in lora_config.h.</t>
+          <t>Measure droop during LoRa TX and sensor bursts. Starting points from BQ25505_DESIGN_INPUTS.md: VCAP_MIN_SENSORS_mV=2700, VCAP_MIN_TX_mV=3000, VCAP_CHARGE_TARGET_mV=3600. Tune on bench.</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">

</xml_diff>